<commit_message>
feat: adiciona conversor de planilhas - transforma qualquer Excel em CSV padrão
</commit_message>
<xml_diff>
--- a/Planilha/Inventário de Bens do Núcleo REI RABINO - Copia.xlsx
+++ b/Planilha/Inventário de Bens do Núcleo REI RABINO - Copia.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SATA INFORMATICA\Desktop\PATRIMONIO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EderD\Desktop\Projetos\Patrimonio do Rei\Patrimonio-do-Rei\Planilha\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_64E4CAD294FAB0F42C8D30D854F0150CBB5DE88A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8445"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cadastro Analítico" sheetId="2" r:id="rId1"/>
     <sheet name="Plan2" sheetId="4" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,6 +28,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -34,12 +37,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>SATA INFORMATICA</author>
   </authors>
   <commentList>
-    <comment ref="D44" authorId="0" shapeId="0">
+    <comment ref="D44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -64,7 +67,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D54" authorId="0" shapeId="0">
+    <comment ref="D54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -1110,7 +1113,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
@@ -1894,7 +1897,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2073,16 +2076,13 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2094,7 +2094,7 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2115,64 +2115,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2202,8 +2151,59 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2242,7 +2242,7 @@
         <xdr:cNvPr id="2" name="Imagem 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE454191-6AB9-4B82-ADB5-A6211BCC2700}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE454191-6AB9-4B82-ADB5-A6211BCC2700}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2550,7 +2550,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA1093"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2594,13 +2594,13 @@
     </row>
     <row r="2" spans="1:27" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
-      <c r="B2" s="96"/>
-      <c r="C2" s="97"/>
-      <c r="D2" s="97"/>
-      <c r="E2" s="97"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="97"/>
-      <c r="H2" s="98"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="80"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
@@ -2624,14 +2624,14 @@
     <row r="3" spans="1:27" ht="81" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5"/>
       <c r="B3" s="6"/>
-      <c r="C3" s="99" t="s">
+      <c r="C3" s="81" t="s">
         <v>235</v>
       </c>
-      <c r="D3" s="100"/>
-      <c r="E3" s="100"/>
-      <c r="F3" s="100"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="101"/>
+      <c r="D3" s="82"/>
+      <c r="E3" s="82"/>
+      <c r="F3" s="82"/>
+      <c r="G3" s="82"/>
+      <c r="H3" s="83"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
@@ -2654,15 +2654,15 @@
     </row>
     <row r="4" spans="1:27" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
-      <c r="B4" s="102" t="s">
+      <c r="B4" s="84" t="s">
         <v>97</v>
       </c>
-      <c r="C4" s="103"/>
-      <c r="D4" s="103"/>
-      <c r="E4" s="103"/>
-      <c r="F4" s="103"/>
-      <c r="G4" s="103"/>
-      <c r="H4" s="104"/>
+      <c r="C4" s="85"/>
+      <c r="D4" s="85"/>
+      <c r="E4" s="85"/>
+      <c r="F4" s="85"/>
+      <c r="G4" s="85"/>
+      <c r="H4" s="86"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
@@ -3053,10 +3053,10 @@
     </row>
     <row r="15" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
-      <c r="B15" s="91" t="s">
+      <c r="B15" s="87" t="s">
         <v>106</v>
       </c>
-      <c r="C15" s="88"/>
+      <c r="C15" s="77"/>
       <c r="D15" s="15"/>
       <c r="E15" s="21">
         <f>SUM(E8:E14)</f>
@@ -3576,7 +3576,7 @@
     </row>
     <row r="29" spans="1:27" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="48"/>
-      <c r="B29" s="67" t="s">
+      <c r="B29" s="66" t="s">
         <v>303</v>
       </c>
       <c r="C29" s="50" t="s">
@@ -4102,7 +4102,7 @@
       <c r="C43" s="15" t="s">
         <v>247</v>
       </c>
-      <c r="D43" s="63">
+      <c r="D43" s="16">
         <v>162</v>
       </c>
       <c r="E43" s="17">
@@ -4490,7 +4490,7 @@
     <row r="54" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="48"/>
       <c r="B54" s="50"/>
-      <c r="C54" s="71"/>
+      <c r="C54" s="70"/>
       <c r="D54" s="53"/>
       <c r="E54" s="51"/>
       <c r="F54" s="18"/>
@@ -4634,10 +4634,10 @@
     </row>
     <row r="59" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5"/>
-      <c r="B59" s="87" t="s">
+      <c r="B59" s="76" t="s">
         <v>106</v>
       </c>
-      <c r="C59" s="88"/>
+      <c r="C59" s="77"/>
       <c r="D59" s="54"/>
       <c r="E59" s="21">
         <f>SUM(E42:E54)</f>
@@ -5197,10 +5197,10 @@
     </row>
     <row r="75" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5"/>
-      <c r="B75" s="87" t="s">
+      <c r="B75" s="76" t="s">
         <v>106</v>
       </c>
-      <c r="C75" s="88"/>
+      <c r="C75" s="77"/>
       <c r="D75" s="54"/>
       <c r="E75" s="21">
         <f>SUM(E61:E74)</f>
@@ -7340,10 +7340,10 @@
     </row>
     <row r="133" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="48"/>
-      <c r="B133" s="67">
+      <c r="B133" s="66">
         <v>160058</v>
       </c>
-      <c r="C133" s="105" t="s">
+      <c r="C133" s="75" t="s">
         <v>332</v>
       </c>
       <c r="D133" s="53"/>
@@ -7412,7 +7412,7 @@
       <c r="A135" s="48"/>
       <c r="B135" s="50"/>
       <c r="C135" s="60"/>
-      <c r="D135" s="69"/>
+      <c r="D135" s="68"/>
       <c r="E135" s="51"/>
       <c r="F135" s="18"/>
       <c r="G135" s="47"/>
@@ -7439,10 +7439,10 @@
     </row>
     <row r="136" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A136" s="48"/>
-      <c r="B136" s="89" t="s">
+      <c r="B136" s="88" t="s">
         <v>106</v>
       </c>
-      <c r="C136" s="90"/>
+      <c r="C136" s="89"/>
       <c r="D136" s="50"/>
       <c r="E136" s="57">
         <f>SUM(E77:E128)</f>
@@ -7473,13 +7473,13 @@
     </row>
     <row r="137" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A137" s="5"/>
-      <c r="B137" s="72" t="s">
+      <c r="B137" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="C137" s="72" t="s">
+      <c r="C137" s="71" t="s">
         <v>112</v>
       </c>
-      <c r="D137" s="73"/>
+      <c r="D137" s="72"/>
       <c r="E137" s="11"/>
       <c r="F137" s="11"/>
       <c r="G137" s="11"/>
@@ -7864,7 +7864,7 @@
       <c r="E148" s="21">
         <v>1160</v>
       </c>
-      <c r="F148" s="70">
+      <c r="F148" s="69">
         <v>46108</v>
       </c>
       <c r="G148" s="16">
@@ -7965,10 +7965,10 @@
     </row>
     <row r="151" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A151" s="5"/>
-      <c r="B151" s="91" t="s">
+      <c r="B151" s="87" t="s">
         <v>106</v>
       </c>
-      <c r="C151" s="88"/>
+      <c r="C151" s="77"/>
       <c r="D151" s="15"/>
       <c r="E151" s="21">
         <f>SUM(E139:E150)</f>
@@ -7999,19 +7999,19 @@
     </row>
     <row r="152" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A152" s="5"/>
-      <c r="B152" s="92" t="s">
+      <c r="B152" s="90" t="s">
         <v>113</v>
       </c>
-      <c r="C152" s="93"/>
+      <c r="C152" s="91"/>
       <c r="D152" s="23" t="s">
         <v>114</v>
       </c>
       <c r="E152" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="F152" s="85"/>
-      <c r="G152" s="85"/>
-      <c r="H152" s="80"/>
+      <c r="F152" s="94"/>
+      <c r="G152" s="94"/>
+      <c r="H152" s="100"/>
       <c r="I152" s="3"/>
       <c r="J152" s="3"/>
       <c r="K152" s="3"/>
@@ -8034,8 +8034,8 @@
     </row>
     <row r="153" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A153" s="5"/>
-      <c r="B153" s="94"/>
-      <c r="C153" s="95"/>
+      <c r="B153" s="92"/>
+      <c r="C153" s="93"/>
       <c r="D153" s="25">
         <v>338</v>
       </c>
@@ -8043,9 +8043,9 @@
         <f>SUM(E151,E136,E75,E59,E40,E30,E15)</f>
         <v>654292.22</v>
       </c>
-      <c r="F153" s="86"/>
-      <c r="G153" s="86"/>
-      <c r="H153" s="81"/>
+      <c r="F153" s="95"/>
+      <c r="G153" s="95"/>
+      <c r="H153" s="101"/>
       <c r="I153" s="3"/>
       <c r="J153" s="3"/>
       <c r="K153" s="3"/>
@@ -8099,13 +8099,13 @@
       <c r="A155" s="28"/>
       <c r="B155" s="3"/>
       <c r="C155" s="29"/>
-      <c r="D155" s="82" t="s">
+      <c r="D155" s="102" t="s">
         <v>116</v>
       </c>
-      <c r="E155" s="83"/>
-      <c r="F155" s="83"/>
-      <c r="G155" s="83"/>
-      <c r="H155" s="84"/>
+      <c r="E155" s="103"/>
+      <c r="F155" s="103"/>
+      <c r="G155" s="103"/>
+      <c r="H155" s="104"/>
       <c r="I155" s="3"/>
       <c r="J155" s="3"/>
       <c r="K155" s="3"/>
@@ -8128,10 +8128,10 @@
     </row>
     <row r="156" spans="1:27" ht="63.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A156" s="28"/>
-      <c r="B156" s="76" t="s">
+      <c r="B156" s="96" t="s">
         <v>221</v>
       </c>
-      <c r="C156" s="77"/>
+      <c r="C156" s="97"/>
       <c r="D156" s="3"/>
       <c r="E156" s="3"/>
       <c r="F156" s="3"/>
@@ -8219,10 +8219,10 @@
     </row>
     <row r="159" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A159" s="28"/>
-      <c r="B159" s="78" t="s">
+      <c r="B159" s="98" t="s">
         <v>234</v>
       </c>
-      <c r="C159" s="79"/>
+      <c r="C159" s="99"/>
       <c r="D159" s="3"/>
       <c r="E159" s="3"/>
       <c r="F159" s="3"/>
@@ -8250,10 +8250,10 @@
     </row>
     <row r="160" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A160" s="28"/>
-      <c r="B160" s="76" t="s">
+      <c r="B160" s="96" t="s">
         <v>250</v>
       </c>
-      <c r="C160" s="77"/>
+      <c r="C160" s="97"/>
       <c r="D160" s="3"/>
       <c r="E160" s="3"/>
       <c r="F160" s="3"/>
@@ -8341,10 +8341,10 @@
     </row>
     <row r="163" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A163" s="28"/>
-      <c r="B163" s="76" t="s">
+      <c r="B163" s="96" t="s">
         <v>251</v>
       </c>
-      <c r="C163" s="77"/>
+      <c r="C163" s="97"/>
       <c r="D163" s="3"/>
       <c r="E163" s="3"/>
       <c r="F163" s="3"/>
@@ -8372,8 +8372,8 @@
     </row>
     <row r="164" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A164" s="28"/>
-      <c r="B164" s="76"/>
-      <c r="C164" s="77"/>
+      <c r="B164" s="96"/>
+      <c r="C164" s="97"/>
       <c r="D164" s="3"/>
       <c r="E164" s="3"/>
       <c r="F164" s="3"/>
@@ -8401,8 +8401,8 @@
     </row>
     <row r="165" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A165" s="28"/>
-      <c r="B165" s="74"/>
-      <c r="C165" s="75" t="s">
+      <c r="B165" s="73"/>
+      <c r="C165" s="74" t="s">
         <v>328</v>
       </c>
       <c r="D165" s="3"/>
@@ -8463,8 +8463,8 @@
     </row>
     <row r="167" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A167" s="28"/>
-      <c r="B167" s="78"/>
-      <c r="C167" s="79"/>
+      <c r="B167" s="98"/>
+      <c r="C167" s="99"/>
       <c r="D167" s="3"/>
       <c r="E167" s="3"/>
       <c r="F167" s="3"/>
@@ -8492,10 +8492,10 @@
     </row>
     <row r="168" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A168" s="28"/>
-      <c r="B168" s="76" t="s">
+      <c r="B168" s="96" t="s">
         <v>117</v>
       </c>
-      <c r="C168" s="77"/>
+      <c r="C168" s="97"/>
       <c r="D168" s="3"/>
       <c r="E168" s="3"/>
       <c r="F168" s="3"/>
@@ -35350,16 +35350,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="C3:H3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="B136:C136"/>
-    <mergeCell ref="B151:C151"/>
-    <mergeCell ref="B152:C153"/>
-    <mergeCell ref="F152:F153"/>
     <mergeCell ref="B164:C164"/>
     <mergeCell ref="B167:C167"/>
     <mergeCell ref="B168:C168"/>
@@ -35370,6 +35360,16 @@
     <mergeCell ref="B160:C160"/>
     <mergeCell ref="B163:C163"/>
     <mergeCell ref="G152:G153"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B136:C136"/>
+    <mergeCell ref="B151:C151"/>
+    <mergeCell ref="B152:C153"/>
+    <mergeCell ref="F152:F153"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B15:C15"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -35379,7 +35379,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -35416,13 +35416,13 @@
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="E3" s="66">
+      <c r="E3" s="65">
         <v>400</v>
       </c>
       <c r="F3" t="s">
         <v>245</v>
       </c>
-      <c r="G3" s="64"/>
+      <c r="G3" s="63"/>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
@@ -35431,14 +35431,14 @@
       <c r="C4">
         <v>1</v>
       </c>
-      <c r="E4" s="66">
+      <c r="E4" s="65">
         <v>350</v>
       </c>
       <c r="F4" t="s">
         <v>262</v>
       </c>
-      <c r="G4" s="64"/>
-      <c r="H4" s="65"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="64"/>
     </row>
     <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
@@ -35447,13 +35447,13 @@
       <c r="C5">
         <v>1</v>
       </c>
-      <c r="E5" s="66">
+      <c r="E5" s="65">
         <v>350</v>
       </c>
       <c r="F5" t="s">
         <v>244</v>
       </c>
-      <c r="G5" s="64"/>
+      <c r="G5" s="63"/>
     </row>
     <row r="6" spans="1:8" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
@@ -35462,13 +35462,13 @@
       <c r="C6">
         <v>1</v>
       </c>
-      <c r="E6" s="66">
+      <c r="E6" s="65">
         <v>400</v>
       </c>
       <c r="F6" t="s">
         <v>245</v>
       </c>
-      <c r="G6" s="64"/>
+      <c r="G6" s="63"/>
     </row>
     <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
@@ -35477,13 +35477,13 @@
       <c r="C7">
         <v>12</v>
       </c>
-      <c r="E7" s="66">
+      <c r="E7" s="65">
         <v>480</v>
       </c>
       <c r="F7" t="s">
         <v>245</v>
       </c>
-      <c r="G7" s="64"/>
+      <c r="G7" s="63"/>
     </row>
     <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
@@ -35492,13 +35492,13 @@
       <c r="C8">
         <v>12</v>
       </c>
-      <c r="E8" s="66">
+      <c r="E8" s="65">
         <v>480</v>
       </c>
       <c r="F8" t="s">
         <v>245</v>
       </c>
-      <c r="G8" s="64"/>
+      <c r="G8" s="63"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
@@ -35507,13 +35507,13 @@
       <c r="C9">
         <v>1</v>
       </c>
-      <c r="E9" s="66">
+      <c r="E9" s="65">
         <v>400</v>
       </c>
       <c r="F9" t="s">
         <v>249</v>
       </c>
-      <c r="G9" s="64"/>
+      <c r="G9" s="63"/>
     </row>
     <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
@@ -35522,13 +35522,13 @@
       <c r="C10">
         <v>1</v>
       </c>
-      <c r="E10" s="66">
+      <c r="E10" s="65">
         <v>299</v>
       </c>
       <c r="F10" t="s">
         <v>249</v>
       </c>
-      <c r="G10" s="64"/>
+      <c r="G10" s="63"/>
     </row>
     <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="15" t="s">
@@ -35537,13 +35537,13 @@
       <c r="C11">
         <v>1</v>
       </c>
-      <c r="E11" s="66">
+      <c r="E11" s="65">
         <v>450</v>
       </c>
       <c r="F11" t="s">
         <v>270</v>
       </c>
-      <c r="G11" s="64"/>
+      <c r="G11" s="63"/>
     </row>
     <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
@@ -35552,13 +35552,13 @@
       <c r="C12">
         <v>1</v>
       </c>
-      <c r="E12" s="66">
+      <c r="E12" s="65">
         <v>400</v>
       </c>
       <c r="F12" t="s">
         <v>279</v>
       </c>
-      <c r="G12" s="64"/>
+      <c r="G12" s="63"/>
     </row>
     <row r="13" spans="1:8" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15" t="s">
@@ -35567,28 +35567,28 @@
       <c r="C13">
         <v>1</v>
       </c>
-      <c r="E13" s="66">
+      <c r="E13" s="65">
         <v>400</v>
       </c>
       <c r="F13" t="s">
         <v>284</v>
       </c>
-      <c r="G13" s="64"/>
+      <c r="G13" s="63"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="68" t="s">
+      <c r="A14" s="67" t="s">
         <v>169</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
-      <c r="E14" s="66">
+      <c r="E14" s="65">
         <v>600</v>
       </c>
       <c r="F14" t="s">
         <v>287</v>
       </c>
-      <c r="G14" s="64"/>
+      <c r="G14" s="63"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>